<commit_message>
Add Kyushu/Okinawa region hospital Excels (Fukuoka/Saga/Nagasaki/Kumamoto/Oita/Kagoshima/Okinawa)
Miyazaki confirmed to have no JRC hospital.

Fix second category shadowing bug: generic "FPD" keyword under
一般撮影（レントゲン） was checked before more specific categories,
mis-labeling items like "X線テレビシステム" or "血管撮影システム"
containing FPD. Reordered CATEGORIES so specific categories are
checked before the generic 一般撮影 fallback, and relabeled affected
rows in previously delivered files (成田, 古河).
</commit_message>
<xml_diff>
--- a/output/古河赤十字病院_随意契約_X線関連.xlsx
+++ b/output/古河赤十字病院_随意契約_X線関連.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>一般撮影（レントゲン）</t>
+          <t>外科用イメージ（可搬型Cアーム透視装置）</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -617,13 +617,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>一般撮影（レントゲン）</t>
+          <t>回診用X線装置</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>公表された随意契約に該当なし</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -662,18 +666,14 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>公表された随意契約に該当なし</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>回診用X線装置</t>
+          <t>一般撮影（レントゲン）</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">

</xml_diff>